<commit_message>
更新基差至 AMS 报告日 2026-10-20：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1515"/>
+  <dimension ref="A1:O1516"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35017,6 +35017,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1516">
+      <c r="A1516" s="1" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1516" t="n">
+        <v>92</v>
+      </c>
+      <c r="C1516" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
更新基差至 AMS 报告日 2026-10-21：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1516"/>
+  <dimension ref="A1:O1517"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35028,6 +35028,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1517">
+      <c r="A1517" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1517" t="n">
+        <v>96</v>
+      </c>
+      <c r="C1517" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
更新基差至 AMS 报告日 2026-10-22：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1517"/>
+  <dimension ref="A1:O1518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35039,6 +35039,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="1518">
+      <c r="A1518" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1518" t="n">
+        <v>96</v>
+      </c>
+      <c r="C1518" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
更新基差至 AMS 报告日 2026-10-23：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1518"/>
+  <dimension ref="A1:O1519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35050,6 +35050,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1519">
+      <c r="A1519" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1519" t="n">
+        <v>96</v>
+      </c>
+      <c r="C1519" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
更新基差至 AMS 报告日 2026-10-26：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1519"/>
+  <dimension ref="A1:O1520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35061,6 +35061,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1520">
+      <c r="A1520" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1520" t="n">
+        <v>96</v>
+      </c>
+      <c r="C1520" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
更新基差至 AMS 报告日 2026-10-28（补 2026-10-27）：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1520"/>
+  <dimension ref="A1:O1522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35072,6 +35072,28 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1521">
+      <c r="A1521" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1521" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="C1521" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1522" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="C1522" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
更新基差至 AMS 报告日 2026-10-29：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1522"/>
+  <dimension ref="A1:O1523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35094,6 +35094,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1523">
+      <c r="A1523" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1523" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="C1523" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
更新基差至 AMS 报告日 2026-10-30：各州 Excel Current+Change 追加，重建 basis_daily 网页。
</commit_message>
<xml_diff>
--- a/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
+++ b/玉米大豆历史数据/大豆基差/Louisiana Basis.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1523"/>
+  <dimension ref="A1:O1524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="14"/>
@@ -35105,6 +35105,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="1524">
+      <c r="A1524" s="1" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1524" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="C1524" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>